<commit_message>
Cập nhật báo cáo Excel trực tuyến
</commit_message>
<xml_diff>
--- a/BaoCao_KAV.xlsx
+++ b/BaoCao_KAV.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Thời gian thống kê: 22/09/2026 13:27 | Nguồn: classroom.khanacademy.org</t>
+          <t>Thời gian thống kê: 22/09/2026 22:32 | Nguồn: classroom.khanacademy.org</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         <v>47</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" s="11" t="n">
         <v>0.1</v>
@@ -795,7 +795,7 @@
         <v>10</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1188,7 +1188,7 @@
         <v>821</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G25" s="15" t="n">
         <v>0.9</v>

</xml_diff>

<commit_message>
Cập nhật báo cáo Excel cả 2 tài khoản THCS & THPT
</commit_message>
<xml_diff>
--- a/BaoCao_KAV.xlsx
+++ b/BaoCao_KAV.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Báo Cáo KAV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng Hợp Toàn Trường" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khối THPT (21 lớp)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khối THCS (12 lớp)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,13 +33,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B365D"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00555555"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -531,6 +533,1234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO THỐNG KÊ TOÀN TRƯỜNG KHAN ACADEMY (KAV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Thời gian thống kê: 17/10/2026 23:04 | Trường: THCS&amp;THPT MONG THỌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Khối / Phân Loại</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Mã Lớp</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tên Lớp Học</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Khóa Học</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Số tài khoản đã tạo</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Đang hoạt động</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Kỹ Năng TB Thành Thạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>GC65CJ23</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>10A1_Năm học 2026-2027_Nguyễn Thị Yến Linh</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>H4S4C7P2</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>10A2_Năm học 2026-2027_Trần Minh Mẫn</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>UWTVBASW</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>10A3_Năm học 2026-2027_Văn Thị Bích Thùy</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>FHGUSN4Z</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>10A4_Năm học 2026-2027_Văn Thị Bích Thùy</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>4NH4T2A4</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>10A5_Năm học 2026-2027_Nguyễn Ngọc Thịnh</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>VZQP4YAF</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>10A6_Năm học 2026-2027_Nguyễn Ngọc Thịnh</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>KMR6W4FR</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>10A7_Năm học 2026-2027_Nguyễn Chí Huy</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>DZWFS5NS</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>10A8_Năm học 2026-2027_Nguyễn Thành Thái</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Toán 10</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>PJP8ZHQ5</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>11A1_Năm học 2026-2027_Nguyễn Ngọc Thịnh</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>UQ77Z4F8</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>11A2_Năm học 2026-2027_Nguyễn Thị Yến Linh</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>6JZUDEYH</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>11A3_Năm Học 2026-2027_Mai Thành Công</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>NFPJ3YUZ</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>11A4_Năm học 2026-2027_Nguyễn Thị Yến Linh</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>EJ5JBTPM</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>11A5_ Năm Học 2026-2027_Nguyễn Ngọc Thịnh</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>N6D6F43M</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>11A6_Năm học 2026-2027_Mai Thành Công</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Toán 11</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Y4KXVHFH</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>12A1-Năm học 2026-2027_Trần Thị Bội Nhung</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>7B39B8FY</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>12A2 - Năm học 2026-2027_Nguyễn Thành Thái</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>2DXNAW8H</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>12A3-Năm học 2026-2027_Mai Thành Công</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>2T2BZU9H</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>12A4-Năm học 2026-2027_Nguyễn Thành Thái</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>MF9R2SND</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>12A5 - Năm học 2026-2027_Trần Thị Bội Nhung</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>BQKUESU3</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>12A6 _Năm học 2026-2027_Nguyễn Thành Thái</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="H24" s="11" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Khối THPT</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Q96EYDVA</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>12A7 - Năm học 2026 - 2027_Trần Thị Bội Nhung</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Toán 12</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>THCS-6A1</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>6A1_Năm học 2026–2027_Lư Ngọc Cẩm</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H26" s="11" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>THCS-6A2</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>6A2_Năm học: 2026–2027_Trần Thị Lý</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>THCS-6A3</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>6A3_Năm học: 2026–2027_Trần Thị Lý</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>THCS-7A1</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>7A1– Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>THCS-7A2</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>7A2– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>THCS-7A3</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>7A3– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>THCS-7A4</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>7A4– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H32" s="11" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>THCS-8A1</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>8A1– 2026–2027– Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>THCS-8A2</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>8A2–Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>THCS-8A3</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>8A3–Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>THCS-9A1</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>9A1– 2026–2027–Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Toán 9</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Khối THCS</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>THCS-9A2</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>9A2–2026–2027–Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Toán 9</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG / TRUNG BÌNH:</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="14" t="n">
+        <v>1424</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>530</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -543,22 +1773,22 @@
     <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BÁO CÁO THỐNG KÊ KỸ NĂNG THÀNH THẠO KHAN ACADEMY (KAV)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>BÁO CÁO KỸ NĂNG THÀNH THẠO KHỐI THPT (TOÁN 10 - 11 - 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Thời gian thống kê: 17/10/2026 22:46 | Nguồn: classroom.khanacademy.org</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="10" customHeight="1"/>
-    <row r="4" ht="28" customHeight="1">
+          <t>Thời gian thống kê: 17/10/2026 23:04 | Trường: THCS&amp;THPT MONG THỌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>STT</t>
@@ -1207,7 +2437,7 @@
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>TỔNG CỘNG / TRUNG BÌNH TOÀN BỘ:</t>
+          <t>TỔNG CỘNG / TRUNG BÌNH:</t>
         </is>
       </c>
       <c r="B26" s="13" t="n"/>
@@ -1231,4 +2461,451 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BÁO CÁO KỸ NĂNG THÀNH THẠO KHỐI THCS (TOÁN 6 - 7 - 8 - 9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Thời gian thống kê: 17/10/2026 23:04 | Trường: THCS&amp;THPT MONG THỌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mã Lớp</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tên Lớp Học</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Khóa Học / Môn</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Số tài khoản đã tạo</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Số tài khoản đang hoạt động</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kỹ Năng TB Thành Thạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>THCS-6A1</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>6A1_Năm học 2026–2027_Lư Ngọc Cẩm</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>THCS-6A2</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>6A2_Năm học: 2026–2027_Trần Thị Lý</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>THCS-6A3</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>6A3_Năm học: 2026–2027_Trần Thị Lý</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Toán 6</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>THCS-7A1</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>7A1– Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>THCS-7A2</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>7A2– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>THCS-7A3</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>7A3– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>THCS-7A4</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>7A4– 2026–2027– Nguyễn Thị Mỹ Trinh</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Toán 7</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>THCS-8A1</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>8A1– 2026–2027– Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>THCS-8A2</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>8A2–Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>THCS-8A3</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>8A3–Đỗ Thị Kim Mai–2026–2027</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Toán 8</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>THCS-9A1</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>9A1– 2026–2027–Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Toán 9</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>THCS-9A2</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>9A2–2026–2027–Nguyễn Thị Thìn</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Toán 9</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG / TRUNG BÌNH:</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="14" t="n">
+        <v>559</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>146</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>